<commit_message>
chore: update WARN dataset
</commit_message>
<xml_diff>
--- a/data/warn_report.xlsx
+++ b/data/warn_report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30203"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30128"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://edd.sharepoint.com/sites/WSB-COWSD-380-PCU/Shared Documents/Website Management/3. Webpage Updates/Layoff Services WARN/2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\WSB-CO\Program Support\WARN\CalJOBS WARN Reports\WARN CALJOBS REPORTS - DAILY\SFY26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{192DC7D3-6F64-4C2E-9447-F5F0BDCA9B89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAE8E07C-F74A-48D0-986A-5F8DE775272D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="751" xr2:uid="{3EA4B9A5-CE9D-4ACF-B45F-4158810915D4}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="751" firstSheet="2" activeTab="2" xr2:uid="{3EA4B9A5-CE9D-4ACF-B45F-4158810915D4}"/>
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="3" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7656" uniqueCount="2584">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7671" uniqueCount="2590">
   <si>
     <t>This worksheet contains 5 sheets. The introductory page, WARN Report Summary, Detailed WARN Report, Call Center Relocations Summary, and Call Center Relocations Report. The second sheet provides an overview of the report according to layoff/closure/relocation types and related quantitative data. The third sheet displays a detailed summary report of affected companies by county. The fourth sheet provides an overview of the report specificially for call center relocations. The fifth sheet displays a detailed summary report of affected companies by county. This Daily WARN Report is updated every Tuesday and Thursday. Hyperlinks to the other 4 sheets can be found below in cell A3-A6.</t>
   </si>
@@ -123,7 +123,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>07/01/25 to 06/10/2026</t>
+      <t>07/01/25 to 06/15/2026</t>
     </r>
     <r>
       <rPr>
@@ -143,7 +143,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>A detailed WARN summary by county and filtered according to processed date. Table Spans cells A2 through I1519.</t>
+      <t>A detailed WARN summary by county and filtered according to processed date. Table Spans cells A2 through I1522.</t>
     </r>
   </si>
   <si>
@@ -7871,6 +7871,24 @@
   </si>
   <si>
     <t>300 Mission Street, 20th Floor  San Francisco CA 94105</t>
+  </si>
+  <si>
+    <t>Hy-Tek Intralogistics</t>
+  </si>
+  <si>
+    <t>11500 Phelan Road  Hesperia CA 92344</t>
+  </si>
+  <si>
+    <t>Leggett &amp; Platt</t>
+  </si>
+  <si>
+    <t>1671 S. Champagne Avenue  Ontario CA 91761</t>
+  </si>
+  <si>
+    <t>Uber Technologies, Inc.</t>
+  </si>
+  <si>
+    <t>1655 3rd Street  San Francisco CA 94158</t>
   </si>
   <si>
     <r>
@@ -7916,7 +7934,7 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-01/01/2023 - 06/10/2026
+01/01/2023 - 06/15/2026
 </t>
     </r>
     <r>
@@ -8279,7 +8297,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -8421,6 +8439,18 @@
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -9214,7 +9244,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1F69E8FD-21FF-4B81-951D-D7EC70F8E5F9}" name="DetailedWarnReport" displayName="DetailedWarnReport" ref="A2:I1519" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1F69E8FD-21FF-4B81-951D-D7EC70F8E5F9}" name="DetailedWarnReport" displayName="DetailedWarnReport" ref="A2:I1522" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{3E60720E-46D7-48F7-AF17-837D42D08A11}" name="County/Parish" dataDxfId="25"/>
     <tableColumn id="2" xr3:uid="{058DED91-D77E-48B6-A71D-06D4A25AA391}" name="Notice_x000a_Date" dataDxfId="24"/>
@@ -9558,12 +9588,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D341DFFF-02D2-4572-95F5-BB3221952133}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="73.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="74" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="130.5">
+    <row r="1" spans="1:1" ht="135">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -9607,13 +9637,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1832896D-8AFB-4FFC-957E-910308F3BC0C}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.5703125" style="3" customWidth="1"/>
     <col min="2" max="2" width="6.42578125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="76.5">
+    <row r="1" spans="1:2" ht="78.75">
       <c r="A1" s="10" t="s">
         <v>6</v>
       </c>
@@ -9632,7 +9662,7 @@
       </c>
       <c r="B3" s="11">
         <f>SUM('Detailed WARN Report '!G:G)</f>
-        <v>78238</v>
+        <v>78566</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -9641,7 +9671,7 @@
       </c>
       <c r="B4" s="11">
         <f>COUNTIF('Detailed WARN Report '!F:F,"Layoff Permanent")</f>
-        <v>1012</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -9668,7 +9698,7 @@
       </c>
       <c r="B7" s="11">
         <f>COUNTIF('Detailed WARN Report '!F:F,"Closure Permanent")</f>
-        <v>396</v>
+        <v>397</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -9700,18 +9730,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3E7117B-AC46-45AC-B2F3-AE611FA82488}">
-  <dimension ref="A1:I1519"/>
-  <sheetFormatPr defaultColWidth="161.42578125" defaultRowHeight="14.45"/>
+  <dimension ref="A1:I1522"/>
+  <sheetFormatPr defaultColWidth="161.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="28.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="66.42578125" style="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="72.85546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.28515625" style="3" customWidth="1"/>
     <col min="7" max="7" width="9.85546875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="54.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="47.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="55.140625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="51.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="22.5703125" customWidth="1"/>
     <col min="11" max="11" width="13.140625" customWidth="1"/>
     <col min="12" max="12" width="12.7109375" customWidth="1"/>
@@ -9719,13 +9749,13 @@
     <col min="14" max="14" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="99.95">
+    <row r="1" spans="1:9" ht="102">
       <c r="A1" s="16" t="s">
         <v>16</v>
       </c>
       <c r="E1" s="3"/>
     </row>
-    <row r="2" spans="1:9" ht="24">
+    <row r="2" spans="1:9" ht="24.75">
       <c r="A2" s="26" t="s">
         <v>17</v>
       </c>
@@ -13640,7 +13670,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="137" spans="1:9">
+    <row r="137" spans="1:9" ht="22.5">
       <c r="A137" s="28" t="s">
         <v>31</v>
       </c>
@@ -30402,7 +30432,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="715" spans="1:9" ht="20.100000000000001">
+    <row r="715" spans="1:9" ht="22.5">
       <c r="A715" s="28" t="s">
         <v>31</v>
       </c>
@@ -47483,7 +47513,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="1304" spans="1:9" ht="20.100000000000001">
+    <row r="1304" spans="1:9" ht="22.5">
       <c r="A1304" s="28" t="s">
         <v>52</v>
       </c>
@@ -47512,7 +47542,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="1305" spans="1:9" ht="20.100000000000001">
+    <row r="1305" spans="1:9" ht="22.5">
       <c r="A1305" s="28" t="s">
         <v>52</v>
       </c>
@@ -47541,7 +47571,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="1306" spans="1:9" ht="20.100000000000001">
+    <row r="1306" spans="1:9" ht="22.5">
       <c r="A1306" s="28" t="s">
         <v>52</v>
       </c>
@@ -53745,6 +53775,93 @@
       </c>
       <c r="I1519" s="31" t="s">
         <v>347</v>
+      </c>
+    </row>
+    <row r="1520" spans="1:9">
+      <c r="A1520" s="50" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1520" s="51">
+        <v>46184</v>
+      </c>
+      <c r="C1520" s="51">
+        <v>46184</v>
+      </c>
+      <c r="D1520" s="51">
+        <v>46244</v>
+      </c>
+      <c r="E1520" s="50" t="s">
+        <v>2578</v>
+      </c>
+      <c r="F1520" s="50" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1520" s="52">
+        <v>200</v>
+      </c>
+      <c r="H1520" s="52" t="s">
+        <v>2579</v>
+      </c>
+      <c r="I1520" s="53" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="1521" spans="1:9">
+      <c r="A1521" s="50" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1521" s="51">
+        <v>46188</v>
+      </c>
+      <c r="C1521" s="51">
+        <v>46188</v>
+      </c>
+      <c r="D1521" s="51">
+        <v>46248</v>
+      </c>
+      <c r="E1521" s="50" t="s">
+        <v>2580</v>
+      </c>
+      <c r="F1521" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1521" s="52">
+        <v>125</v>
+      </c>
+      <c r="H1521" s="52" t="s">
+        <v>2581</v>
+      </c>
+      <c r="I1521" s="53" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="1522" spans="1:9">
+      <c r="A1522" s="50" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1522" s="51">
+        <v>46185</v>
+      </c>
+      <c r="C1522" s="51">
+        <v>46188</v>
+      </c>
+      <c r="D1522" s="51">
+        <v>46245</v>
+      </c>
+      <c r="E1522" s="50" t="s">
+        <v>2582</v>
+      </c>
+      <c r="F1522" s="50" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1522" s="52">
+        <v>3</v>
+      </c>
+      <c r="H1522" s="52" t="s">
+        <v>2583</v>
+      </c>
+      <c r="I1522" s="53" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -53761,7 +53878,7 @@
           <x14:formula1>
             <xm:f>'Industry List'!$A$1:$A$22</xm:f>
           </x14:formula1>
-          <xm:sqref>I3:I1519</xm:sqref>
+          <xm:sqref>I3:I1522</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -53772,15 +53889,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CC03875-3DF4-4258-8762-7FFE2A7D620D}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" style="22" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.7109375" style="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="95.1">
+    <row r="1" spans="1:2" ht="97.5">
       <c r="A1" s="1" t="s">
-        <v>2578</v>
+        <v>2584</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -53868,25 +53985,25 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EE76718-798E-45ED-8CA1-01AA760CE5F1}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.140625" style="18" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.5703125" style="18" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" style="18" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" customWidth="1"/>
+    <col min="2" max="2" width="8.42578125" style="18" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" style="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" style="18" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="31.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="34.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="98.45">
+    <row r="1" spans="1:8" ht="99.75">
       <c r="A1" s="25" t="s">
-        <v>2579</v>
+        <v>2585</v>
       </c>
       <c r="E1"/>
     </row>
-    <row r="2" spans="1:8" ht="24">
+    <row r="2" spans="1:8" ht="24.75">
       <c r="A2" s="19" t="s">
         <v>17</v>
       </c>
@@ -53926,7 +54043,7 @@
         <v>45047</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>2580</v>
+        <v>2586</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>54</v>
@@ -53949,7 +54066,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E81B0C9-EE0D-4672-99B4-ACA7D2D31E92}">
   <dimension ref="A1:A22"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="67.28515625" bestFit="1" customWidth="1"/>
   </cols>
@@ -53966,7 +54083,7 @@
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>2581</v>
+        <v>2587</v>
       </c>
     </row>
     <row r="4" spans="1:1">
@@ -54056,12 +54173,12 @@
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>2582</v>
+        <v>2588</v>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" t="s">
-        <v>2583</v>
+        <v>2589</v>
       </c>
     </row>
   </sheetData>
@@ -54070,17 +54187,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="9ac7e9dd-8d2d-4750-b54a-f534515ac3a2" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="82b749e3-8208-459a-bfc0-9b428d09cbab">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -54089,7 +54195,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E614ED5C53901F4C88FF6AEBBF3D8E0D" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="529ed3825ab478a5ffdc44eb265dc6f5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="82b749e3-8208-459a-bfc0-9b428d09cbab" xmlns:ns3="9ac7e9dd-8d2d-4750-b54a-f534515ac3a2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b7c2030912f9588e16c624efbe24e62a" ns2:_="" ns3:_="">
     <xsd:import namespace="82b749e3-8208-459a-bfc0-9b428d09cbab"/>
@@ -54296,16 +54402,27 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="9ac7e9dd-8d2d-4750-b54a-f534515ac3a2" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="82b749e3-8208-459a-bfc0-9b428d09cbab">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{003C8481-1A20-4EFB-B5FE-803A2EDAB8F7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E685C52-A6E2-47A3-B296-630123D79679}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D5EB3E32-C54D-49D1-86F5-AD55C5FB43B9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{92D1B9B6-2C55-4A38-8AC5-6016FD477CCF}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9EC50D9-E8AD-45D0-AAAA-B1B0DE75EBF3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58D11D8A-B943-4ACE-951B-4E94023D0688}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>